<commit_message>
chore: bump project-09 submodule (WS0 reorg) + update 电器元件采购.xlsx
- project-09: 6cb8c9b..b4c6a40 (assignments/WorkSheet WS0 reorg + ESP32-C3 Blink EN docx)
- 电器元件采购.xlsx: procurement spreadsheet update
</commit_message>
<xml_diff>
--- a/电器元件采购.xlsx
+++ b/电器元件采购.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding\Summer_project\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7FE8C1-251A-438B-A4B8-CD86D705E184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="4440" yWindow="4440" windowWidth="21600" windowHeight="13210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,15 +24,226 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+  <si>
+    <t>商品名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>数量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>链接</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10种规格200个 整流二极管套装 1N4001-1N4007 1N5817-1N5819现货-淘宝网</t>
+  </si>
+  <si>
+    <t>整流二极管套装</t>
+  </si>
+  <si>
+    <t>5个IRLB8721 IRLB8721PBF 62A/30V MOS场效应管TO-220全新原装-淘宝网</t>
+  </si>
+  <si>
+    <t>NMOS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5*2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.54MM间距 单排针 双排针 全铜镀金1U 3U 高品质 高度11.3 直针-tmall.com天猫</t>
+  </si>
+  <si>
+    <t>单排50条</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>排针公座</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>排针母座</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1x22p 2.54MM直插单排母黑色 10个</t>
+  </si>
+  <si>
+    <t>双排母2.54mm单排母排针母座排座针插座插针2.0 1/2/3/4/6/10-40P-tmall.com天猫</t>
+  </si>
+  <si>
+    <t>价格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>实验室电感套装</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>实验室电容套装</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>实验室电阻套装</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>0510</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF5000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>系列</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF5000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF5000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>种型号各</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF5000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF5000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>个</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0510色码电感包1W色环电感包电子样品包10种/16种/25种感量各10只-淘宝网</t>
+  </si>
+  <si>
+    <t>1/4W电阻41种每种20只共820只(盒装)</t>
+  </si>
+  <si>
+    <t>盒装1/4w金属膜电阻包 精度1% 30种常用直插五色环电阻包 共600只-tmall.com天猫</t>
+  </si>
+  <si>
+    <t>450V68UF 18X25 KXG 10个</t>
+  </si>
+  <si>
+    <t>450V68UF 18X25 KXG 全新日本黑金刚 68uF 450V 高频低阻电解电容-淘宝网</t>
+  </si>
+  <si>
+    <t>函数信号发生器</t>
+  </si>
+  <si>
+    <t>FY6900-50M 采样率250MSa</t>
+  </si>
+  <si>
+    <t>函数信号发生器FY6900双通道20Mdds任意波形多功能脉冲频率计数器-淘宝网</t>
+  </si>
+  <si>
+    <t>入门套件UNO</t>
+  </si>
+  <si>
+    <t>入门套件UNO R3迷你面包板LED跳线电线按钮 用于zarduino Diy套件-淘宝网</t>
+  </si>
+  <si>
+    <t>买标准款</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>吸烟仪 烙铁焊接排烟仪小型焊锡抽烟机风扇活性碳过滤 台式净化器-淘宝网</t>
+  </si>
+  <si>
+    <t>蜂侠吸烟仪-7叶</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="PingFang SC"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFFF5000"/>
+      <name val="PingFang SC"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFFF5000"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFFF5000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="PingFang SC"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,14 +263,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +556,183 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="23.75" customWidth="1"/>
+    <col min="2" max="2" width="20.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>12.2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>5.5</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>7.5</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>86</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="14.5">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7">
+        <v>13.8</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10">
+        <v>667</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <v>5.8</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="https://item.taobao.com/item.htm?abbucket=17&amp;id=566898578778&amp;mi_id=00001eEMkiAR6YgYCiKLBc652FK9SwxJXmWMusTs8Yz8Bk4&amp;ns=1&amp;spm=a21n57.1.hoverItem.8&amp;utparam=%7B%22aplus_abtest%22%3A%220095c96ba1801467e7b6b21387a68cda%22%7D&amp;xxc=taobaoSearch" xr:uid="{ABA24B84-790E-4546-A4C7-EB029EFC692E}"/>
+    <hyperlink ref="D3" r:id="rId2" display="https://item.taobao.com/item.htm?abbucket=17&amp;id=928067516145&amp;mi_id=0000BJ3L4T-LFV46NWqZWo_9f5BrxHidk29VktpjawvyEkE&amp;ns=1&amp;skuId=5976509555411&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%223fa7802e6a293061dd92cf1c3c59eadf%22%7D&amp;xxc=taobaoSearch" xr:uid="{56E875DB-3B19-4640-B747-10928D978AE0}"/>
+    <hyperlink ref="D4" r:id="rId3" display="https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1105809537%3AN%3AYhZ9BCTMjCVmm%2BrIrbS2bg%3D%3D%3Ada8403d8fdd51fc7ce24185f11156dc3&amp;ali_trackid=1_da8403d8fdd51fc7ce24185f11156dc3&amp;id=520519446085&amp;mi_id=0000oYrwAg0-1xVPA6xlwDGbACQbYw2Jeoxv1-mh5Ryemns&amp;mm_sceneid=1_0_44278350_0&amp;skuId=3102460202027&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%22348df709f078ef110a846bd7c8677375%22%7D&amp;xxc=ad_ztc" xr:uid="{D73E8301-FDDB-4133-AA47-28D54970A55F}"/>
+    <hyperlink ref="D5" r:id="rId4" display="https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1104520036%3AH%3Asoi9kAuGO2sdjZOCZxIcSA%3D%3D%3A72cfc2b94f336c8ae4ed19bf535358d2&amp;ali_trackid=318_72cfc2b94f336c8ae4ed19bf535358d2&amp;id=13321689910&amp;mi_id=0000ucJEyk7O9pBhcoh_1G3irXc_YDx22tANZGeWGs4CGwk&amp;mm_sceneid=0_0_28706210_0&amp;priceTId=214783a717837600320204087e0e4a&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%2275974f453f88062496ad286b9e3f8b35%22%7D&amp;xxc=ad_ztc&amp;skuId=3632078798041" xr:uid="{96996BB1-6B34-4343-B594-1E482A99480E}"/>
+    <hyperlink ref="D7" r:id="rId5" display="https://item.taobao.com/item.htm?abbucket=17&amp;id=634108812292&amp;mi_id=0000vjITOthjfjde0zgP28cAQliBmvnfU_3I8aDLR7l_zHY&amp;ns=1&amp;priceTId=2150444517837888472328755e1192&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%227b0ab995cf25e3ba6ee273252ba30fae%22%7D&amp;xxc=taobaoSearch" xr:uid="{7BEFCE74-C32F-4EE5-B806-B444BD089216}"/>
+    <hyperlink ref="D9" r:id="rId6" display="https://detail.tmall.com/item.htm?abbucket=17&amp;id=673861210166&amp;mi_id=0000p1k_e0Y34QgZrtNPRrMRq2ZjHbXrpi7-uQ-TOnk4YUw&amp;ns=1&amp;priceTId=2150444517837891437773452e1192&amp;spm=a21n57.1.hoverItem.4&amp;utparam=%7B%22aplus_abtest%22%3A%22fb18630e4c12cbc170214235c54cce39%22%7D&amp;xxc=taobaoSearch" xr:uid="{162CF17E-6380-419A-872A-1500247C58EF}"/>
+    <hyperlink ref="D8" r:id="rId7" display="https://item.taobao.com/item.htm?ali_refid=a3_430582_1006%3A2620756681%3AH%3AkLjBTGamWExgt36wmTyEmQ%3D%3D%3Ad73971580530859c7b97da5ddbc44df1&amp;ali_trackid=282_d73971580530859c7b97da5ddbc44df1&amp;id=954846790591&amp;mi_id=0000zZeZZ-n9cS9qo_CqmFbJ2QZZLFq6UAZQ1w8hHuG2ipk&amp;mm_sceneid=1_0_7772506767_0&amp;priceTId=214780e217837898175918620e0f93&amp;skuId=6276490083949&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%229e870264409ee9a97f7b8cd7f5451b55%22%7D&amp;xxc=ad_ztc" xr:uid="{51882A03-20A4-44B8-BDB2-514D9123E0FE}"/>
+    <hyperlink ref="D10" r:id="rId8" display="https://item.taobao.com/item.htm?abbucket=17&amp;id=799038688099&amp;mi_id=0000-h5ZvMa2oL2pmlbmY1VPT3g9KFWJ_QC7qZ99awi0whw&amp;ns=1&amp;priceTId=2147823a17838256963511015e116a&amp;spm=a21n57.1.item.4&amp;utparam=%7B%22aplus_abtest%22%3A%2219b672d9b0d216a31c8e758cde5c9dfa%22%7D&amp;xxc=taobaoSearch&amp;skuId=5615491103735" xr:uid="{A6C77A07-CC1B-42D0-8A8B-03BAABB5C671}"/>
+    <hyperlink ref="D11" r:id="rId9" display="https://item.taobao.com/item.htm?abbucket=17&amp;id=595447129463&amp;mi_id=0000Dhd99754rau0itt9J05vDxUGiboFzPPA3N2V1uHZ-IE&amp;ns=1&amp;priceTId=2150459a17838285986833831e110b&amp;spm=a21n57.1.hoverItem.6&amp;utparam=%7B%22aplus_abtest%22%3A%22fe493c3497eca3cae359d3d02dafec9b%22%7D&amp;xxc=taobaoSearch" xr:uid="{638A10C8-5C25-404F-B6B0-5194761B4023}"/>
+    <hyperlink ref="D6" r:id="rId10" display="https://item.taobao.com/item.htm?id=647899559075&amp;last_time=1783832715&amp;mi_id=0000GigVe0lDc3DbXvdSdrCrZsDqlh_IVpRen2ecRnG7kvQ&amp;scm=1007.13982.82927.0&amp;spm=tbpc.mytb_footmark.item.goods&amp;upStreamPrice=7400&amp;skuId=4665984884316" xr:uid="{73270066-2151-442B-B3C8-F7FE52EF5AAE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>